<commit_message>
data: update 2026-06-18 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/daily_logs/daily_2026-06-18.xlsx
+++ b/daily_logs/daily_2026-06-18.xlsx
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Steepening</t>
+          <t>Bull Steepening</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>88</v>
+        <v>73</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.14</v>
+        <v>2.23</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-1</v>
+        <v>-5</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,7 +1064,7 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.43</v>
+        <v>4.49</v>
       </c>
       <c r="F19" s="24" t="n">
         <v>18</v>
@@ -1096,7 +1096,7 @@
         <v>4.93</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.26</v>
+        <v>2.25</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.21</v>
+        <v>2.23</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1657,7 +1657,7 @@
         <v>-2</v>
       </c>
       <c r="F39" s="24" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
@@ -1690,7 +1690,7 @@
         <v>0</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>-12</v>
+        <v>-11</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1886,10 +1886,10 @@
         </is>
       </c>
       <c r="E47" s="24" t="n">
-        <v>3080.72</v>
+        <v>3033.44</v>
       </c>
       <c r="F47" s="24" t="n">
-        <v>-125.82</v>
+        <v>-131.84</v>
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>271</v>
+        <v>263</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2471,10 +2471,10 @@
         </is>
       </c>
       <c r="E66" s="24" t="n">
-        <v>6.52</v>
+        <v>6.47</v>
       </c>
       <c r="F66" s="24" t="n">
-        <v>-43</v>
+        <v>-37</v>
       </c>
       <c r="G66" s="6" t="n"/>
     </row>
@@ -2914,8 +2914,8 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=9.0bp [OK]
-HY OAS 5dd=7.0bp
+          <t>HY OAS 20dd=15.0bp [OK]
+HY OAS 5dd=17.0bp
 HYG 5d=0.3% [OK]
 HYG DD%=None% max drawdown
 FXY 5d=-0.1% [OK]

</xml_diff>